<commit_message>
feat(core)!: Changed the behavior of shift type requirements containing shift type groups
Originally `ALL` -> `[[D], [E], [N]]`, now `ALL` -> `[[D, E, N]]`
</commit_message>
<xml_diff>
--- a/core/tests/testcases/basics/03_4nurses_3shifts_7days_shift_type_requirement_shift_type_all.prettify.xlsx
+++ b/core/tests/testcases/basics/03_4nurses_3shifts_7days_shift_type_requirement_shift_type_all.prettify.xlsx
@@ -552,81 +552,25 @@
       <c r="A4" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="H4" s="1" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="1" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="B5" s="4" t="inlineStr"/>
+      <c r="C5" s="4" t="inlineStr"/>
+      <c r="D5" s="4" t="inlineStr"/>
+      <c r="E5" s="4" t="inlineStr"/>
+      <c r="F5" s="4" t="inlineStr"/>
+      <c r="G5" s="4" t="inlineStr"/>
+      <c r="H5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -635,7 +579,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="2" t="inlineStr"/>

</xml_diff>